<commit_message>
fix: add support for COUNTA, COUNTBLANK, and other extended Excel functions
</commit_message>
<xml_diff>
--- a/templates/DEPT_EMPLOYEES.xlsx
+++ b/templates/DEPT_EMPLOYEES.xlsx
@@ -1,67 +1,115 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\ApexReports\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12450"/>
   </bookViews>
   <sheets>
-    <sheet name="Departments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Departments" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+  <si>
+    <t>{{#each departments page_break=true}}</t>
+  </si>
+  <si>
+    <t>DEPARTMENT: {{dept_name}} (Location: {{loc}})</t>
+  </si>
+  <si>
+    <t>Emp No</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
+  </si>
+  <si>
+    <t>Job Title</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>{{#each employees}}</t>
+  </si>
+  <si>
+    <t>{{empno}}</t>
+  </si>
+  <si>
+    <t>{{ename}}</t>
+  </si>
+  <si>
+    <t>{{job}}</t>
+  </si>
+  <si>
+    <t>{{sal}}</t>
+  </si>
+  <si>
+    <t>{{/each}}</t>
+  </si>
+  <si>
+    <t>Department Total:</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF334155"/>
       <name val="Calibri"/>
-      <color rgb="00334155"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
-        <bgColor rgb="00E2E8F0"/>
+        <fgColor rgb="FFE2E8F0"/>
+        <bgColor rgb="FFE2E8F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F172A"/>
-        <bgColor rgb="000F172A"/>
+        <fgColor rgb="FF0F172A"/>
+        <bgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,87 +125,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -445,111 +446,94 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>{{#each departments page_break=true}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>DEPARTMENT: {{dept_name}} (Location: {{loc}})</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Emp No</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Employee Name</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Job Title</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Salary</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>{{#each employees}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>{{empno}}</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>{{ename}}</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>{{job}}</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>{{sal}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>{{/each}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Department Total:</t>
-        </is>
-      </c>
-      <c r="D7" s="6">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f>COUNTA(A5:A5)</f>
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="8">
         <f>SUM(D5:D5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>{{/each}}</t>
-        </is>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: correctly handle merged cells inside repeating blocks without overlapping previous iterations
</commit_message>
<xml_diff>
--- a/templates/DEPT_EMPLOYEES.xlsx
+++ b/templates/DEPT_EMPLOYEES.xlsx
@@ -512,10 +512,6 @@
       <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <f>COUNTA(A5:A5)</f>
-        <v>1</v>
-      </c>
       <c r="C7" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
feat: enforce CSS page breaks in HTML preview and browser PDF generation
</commit_message>
<xml_diff>
--- a/templates/DEPT_EMPLOYEES.xlsx
+++ b/templates/DEPT_EMPLOYEES.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>{{#each departments page_break=true}}</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>Department Total:</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>{{manager}}</t>
   </si>
 </sst>
 </file>
@@ -130,12 +136,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -144,6 +144,10 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -447,32 +451,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="4" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -485,13 +491,16 @@
       <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -501,34 +510,38 @@
       <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="7"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="6">
         <f>SUM(D5:D5)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(docker): add chromium to Dockerfile and add .dockerignore for clean builds
</commit_message>
<xml_diff>
--- a/templates/DEPT_EMPLOYEES.xlsx
+++ b/templates/DEPT_EMPLOYEES.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>{{#each departments page_break=true}}</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>{{manager}}</t>
+  </si>
+  <si>
+    <t>a</t>
   </si>
 </sst>
 </file>
@@ -451,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -539,6 +542,11 @@
         <v>11</v>
       </c>
     </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>